<commit_message>
[NCBI Daily] 2026-08-07 pipeline results
</commit_message>
<xml_diff>
--- a/results/2026-08-07/NCBI_Eukaryota_Taxonomy_Summary.xlsx
+++ b/results/2026-08-07/NCBI_Eukaryota_Taxonomy_Summary.xlsx
@@ -466,10 +466,10 @@
         <v>1189</v>
       </c>
       <c r="E2" t="n">
-        <v>41983</v>
+        <v>41984</v>
       </c>
       <c r="F2" t="n">
-        <v>766043</v>
+        <v>766060</v>
       </c>
     </row>
     <row r="3">
@@ -490,10 +490,10 @@
         <v>482</v>
       </c>
       <c r="E3" t="n">
-        <v>14559</v>
+        <v>14553</v>
       </c>
       <c r="F3" t="n">
-        <v>274708</v>
+        <v>280644</v>
       </c>
     </row>
     <row r="4">
@@ -514,10 +514,10 @@
         <v>647</v>
       </c>
       <c r="E4" t="n">
-        <v>5330</v>
+        <v>5332</v>
       </c>
       <c r="F4" t="n">
-        <v>77339</v>
+        <v>77421</v>
       </c>
     </row>
     <row r="5">
@@ -538,10 +538,10 @@
         <v>187</v>
       </c>
       <c r="E5" t="n">
-        <v>1637</v>
+        <v>1639</v>
       </c>
       <c r="F5" t="n">
-        <v>56329</v>
+        <v>56330</v>
       </c>
     </row>
     <row r="6">
@@ -589,7 +589,7 @@
         <v>1744</v>
       </c>
       <c r="F7" t="n">
-        <v>41615</v>
+        <v>41616</v>
       </c>
     </row>
     <row r="8">
@@ -613,7 +613,7 @@
         <v>3502</v>
       </c>
       <c r="F8" t="n">
-        <v>32390</v>
+        <v>32392</v>
       </c>
     </row>
     <row r="9">
@@ -637,7 +637,7 @@
         <v>4083</v>
       </c>
       <c r="F9" t="n">
-        <v>32068</v>
+        <v>32070</v>
       </c>
     </row>
     <row r="10">
@@ -661,7 +661,7 @@
         <v>1645</v>
       </c>
       <c r="F10" t="n">
-        <v>25060</v>
+        <v>25064</v>
       </c>
     </row>
     <row r="11">
@@ -733,7 +733,7 @@
         <v>1217</v>
       </c>
       <c r="F13" t="n">
-        <v>14600</v>
+        <v>14601</v>
       </c>
     </row>
     <row r="14">
@@ -1093,7 +1093,7 @@
         <v>23</v>
       </c>
       <c r="F28" t="n">
-        <v>6412</v>
+        <v>6413</v>
       </c>
     </row>
     <row r="29">
@@ -1357,7 +1357,7 @@
         <v>395</v>
       </c>
       <c r="F39" t="n">
-        <v>3193</v>
+        <v>3194</v>
       </c>
     </row>
     <row r="40">
@@ -1693,7 +1693,7 @@
         <v>123</v>
       </c>
       <c r="F53" t="n">
-        <v>2260</v>
+        <v>2261</v>
       </c>
     </row>
     <row r="54">
@@ -2053,7 +2053,7 @@
         <v>67</v>
       </c>
       <c r="F68" t="n">
-        <v>1241</v>
+        <v>1253</v>
       </c>
     </row>
     <row r="69">
@@ -2491,22 +2491,22 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Mortierellomycota</t>
+          <t>Streptophyta</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Mortierellomycetes</t>
+          <t>Pinopsida</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D87" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="F87" t="n">
         <v>858</v>
@@ -2515,25 +2515,25 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Streptophyta</t>
+          <t>Mortierellomycota</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Pinopsida</t>
+          <t>Mortierellomycetes</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D88" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E88" t="n">
-        <v>74</v>
+        <v>20</v>
       </c>
       <c r="F88" t="n">
-        <v>857</v>
+        <v>858</v>
       </c>
     </row>
     <row r="89">
@@ -2821,7 +2821,7 @@
         <v>55</v>
       </c>
       <c r="F100" t="n">
-        <v>530</v>
+        <v>531</v>
       </c>
     </row>
     <row r="101">

</xml_diff>